<commit_message>
CDISC --DY convention, BMIBLGR1 missing guard, TRTSDTM datetime, e8601da informat
</commit_message>
<xml_diff>
--- a/adam_spec_full.xlsx
+++ b/adam_spec_full.xlsx
@@ -3431,7 +3431,7 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>RANDDT - SCRPDT + 1. Missing if either date is missing.</t>
+          <t>(RANDDT - SCRPDT) + (RANDDT &gt;= SCRPDT). Missing if either date is missing. Uses CDISC --DY convention (no day 0).</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>DTHDT - TRTSDT + 1. Missing if either date is missing.</t>
+          <t>(DTHDT - TRTSDT) + (DTHDT &gt;= TRTSDT). Missing if either date is missing. Uses CDISC --DY convention (no day 0).</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>EOSDT - TRTSDT + 1. Missing if either date is missing.</t>
+          <t>(EOSDT - TRTSDT) + (EOSDT &gt;= TRTSDT). Missing if either date is missing. Uses CDISC --DY convention (no day 0).</t>
         </is>
       </c>
     </row>

</xml_diff>